<commit_message>
Update Hindi questionnaire and audio files
</commit_message>
<xml_diff>
--- a/Hindi 24 sentences.xlsx
+++ b/Hindi 24 sentences.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7ba77bf8d4b5edec/Desktop/IIITH DOCUMENTS/prosody_questionnaire/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{44433301-E5AE-42B2-AC9E-2D20BA14D5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F03BCFB-37AF-48DB-9CD1-1CA3791C23E3}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="8_{44433301-E5AE-42B2-AC9E-2D20BA14D5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C419E43-68ED-4615-8472-FFD69EB7ED17}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="136">
   <si>
     <t>sample id</t>
   </si>
@@ -118,51 +118,9 @@
     <t>QijH4UAqGD8_sentence_00909.m4a</t>
   </si>
   <si>
-    <t>v21</t>
-  </si>
-  <si>
-    <t>But that's all it was.</t>
-  </si>
-  <si>
-    <t>पर यही सब था​.</t>
-  </si>
-  <si>
-    <t>लेकिन यह सब था.</t>
-  </si>
-  <si>
-    <t>eaCrsBtiYA4_sentence_01283.m4a</t>
-  </si>
-  <si>
-    <t>It's all in English."</t>
-  </si>
-  <si>
-    <t>वो तो पूरा ही अंग्रेजी में है।"</t>
-  </si>
-  <si>
-    <t>यह सब अंग्रेजी में है".</t>
-  </si>
-  <si>
-    <t>tFX68SJs2-0_sentence_01541.m4a</t>
-  </si>
-  <si>
-    <t>Where do we even begin with that insight?</t>
-  </si>
-  <si>
-    <t>इस समझ की शुरुआत भी कहाँ से करें?</t>
-  </si>
-  <si>
-    <t>हम उस अंतर्दृष्टि से कहाँ से शुरू करें?</t>
-  </si>
-  <si>
-    <t>even</t>
-  </si>
-  <si>
     <t>भी</t>
   </si>
   <si>
-    <t>MB5IX-np5fE_sentence_01018.m4a</t>
-  </si>
-  <si>
     <t>We just happen to make great computers.</t>
   </si>
   <si>
@@ -178,21 +136,6 @@
     <t>qp0HIF3SfI4_sentence_01085.m4a</t>
   </si>
   <si>
-    <t>I also thought, isn't this kind of obvious?</t>
-  </si>
-  <si>
-    <t>मैंने यह भी सोचा, क्या यह स्पष्ट नहीं है?</t>
-  </si>
-  <si>
-    <t>मैंने सोचा, क्या यह स्पष्ट नहीं है?</t>
-  </si>
-  <si>
-    <t>also</t>
-  </si>
-  <si>
-    <t>MB5IX-np5fE_sentence_01098.m4a</t>
-  </si>
-  <si>
     <t>In fact, some of his ideas were bad.</t>
   </si>
   <si>
@@ -271,21 +214,6 @@
     <t>lmyZMtPVodo_sentence_00630.m4a</t>
   </si>
   <si>
-    <t>But now Web video has made it so that any of us or any of the creative things that we do can become completely famous in a part of our world's culture.</t>
-  </si>
-  <si>
-    <t>अब तो वेब विडियो ने ऐसा कर दिया है कि हम में से कोई भी, या हमारी कोई भी रचनात्मक चीज़ बहुत ही मशहूर हो सकती है, हमारी दुनिया की संस्कृति का हिस्सा हो सकती है।</t>
-  </si>
-  <si>
-    <t>लेकिन अब वेब वीडियो ने इसे ऐसा बना दिया है कि हममें से कोई भी या जो भी रचनात्मक काम हम करते हैं वह पूरी तरह से हमारे विश्व की संस्कृति के एक हिस्से में प्रसिद्ध हो सकता है।</t>
-  </si>
-  <si>
-    <t>now</t>
-  </si>
-  <si>
-    <t>BpxVIwCbBK0_sentence_00724.m4a</t>
-  </si>
-  <si>
     <t>And by "why" I don't mean "to make a profit." That's a result. It's always a result.</t>
   </si>
   <si>
@@ -331,21 +259,6 @@
     <t>RcGyVTAoXEU_sentence_01243.m4a</t>
   </si>
   <si>
-    <t>So David, in that story, is supposed to be the underdog, right?</t>
-  </si>
-  <si>
-    <t>तो इस कहानी में डेविड कम क्षमता का व्यक्ति है,है ना?</t>
-  </si>
-  <si>
-    <t>तो डेविड, उस कहानी में, है कि underdog होना चाहिए, सही है?</t>
-  </si>
-  <si>
-    <t>right?</t>
-  </si>
-  <si>
-    <t>ziGD7vQOwl8_sentence_02560.m4a</t>
-  </si>
-  <si>
     <t>Is this what you wanted?</t>
   </si>
   <si>
@@ -394,21 +307,9 @@
     <t>सभी का कल्याण करना, यह तो समुदाय का काम है।</t>
   </si>
   <si>
-    <t>पर यह सब था​.</t>
-  </si>
-  <si>
-    <t>वो तो पूरा अंग्रेजी में है।"</t>
-  </si>
-  <si>
-    <t>इस समझ की शुरुआत कहाँ से करें?</t>
-  </si>
-  <si>
     <t>हम बढ़िया कंप्यूटर बनाते हैं.</t>
   </si>
   <si>
-    <t>मैंने यह सोचा, क्या यह स्पष्ट नहीं है?</t>
-  </si>
-  <si>
     <t>वास्तव में उनके कुछ विचार गलत थे.</t>
   </si>
   <si>
@@ -424,9 +325,6 @@
     <t>मेरा पहला निष्कर्ष यह था कि वे बेहतर लोग हैं.</t>
   </si>
   <si>
-    <t>अब वेब विडियो ने ऐसा कर दिया है कि हम में से कोई भी, या हमारी कोई भी रचनात्मक चीज़ बहुत ही मशहूर हो सकती है, हमारी दुनिया की संस्कृति का हिस्सा हो सकती है।</t>
-  </si>
-  <si>
     <t>और इस “क्यों” का हेतु “लाभ कमाना” नहीं है. वह तो परिणाम है . यह सदा परिणाम है</t>
   </si>
   <si>
@@ -436,13 +334,100 @@
     <t xml:space="preserve">आपको गिनती नही आती अच्छी तरहसे है </t>
   </si>
   <si>
-    <t>तो इस कहानी में डेविड कम क्षमता का व्यक्ति है</t>
-  </si>
-  <si>
     <t xml:space="preserve">तुम यही चाहते थे </t>
   </si>
   <si>
     <t xml:space="preserve">तुम ने मुझे पहचाना नहीं है </t>
+  </si>
+  <si>
+    <t>I find foreign languages very interesting.</t>
+  </si>
+  <si>
+    <t>very</t>
+  </si>
+  <si>
+    <t>मेरे ख़याल से विदेशी भाषाएँ बहुत ही दिलचस्प होतीं हैं।</t>
+  </si>
+  <si>
+    <t>मेरे ख़याल से विदेशी भाषाएँ बहुत दिलचस्प होतीं हैं।</t>
+  </si>
+  <si>
+    <t>That child is only four, but he can already count to 100.</t>
+  </si>
+  <si>
+    <t>वह बच्चा हालांकि केवल चार साल का ही है, वह अभी से ही सौ तक गिनती कर सकता है।</t>
+  </si>
+  <si>
+    <t>वह बच्चा हालांकि केवल चार साल का है, वह अभी से ही सौ तक गिनती कर सकता है।</t>
+  </si>
+  <si>
+    <t>only four</t>
+  </si>
+  <si>
+    <t>वह बच्चा केवल चार साल का है, लेकिन वह पहले से ही 100 तक गिन सकता है।</t>
+  </si>
+  <si>
+    <t>Don't drink any alcohol.</t>
+  </si>
+  <si>
+    <t>शराब की एक बूंद भी मत पियो।</t>
+  </si>
+  <si>
+    <t>शराब की एक बूंद मत पियो।</t>
+  </si>
+  <si>
+    <t>शराब का सेवन बिल्कुल न करें।</t>
+  </si>
+  <si>
+    <t>any alcohol</t>
+  </si>
+  <si>
+    <t>There weren't any children in the park yesterday.</t>
+  </si>
+  <si>
+    <t>कल पार्क में एक भी बच्चा नहीं था।</t>
+  </si>
+  <si>
+    <t>कल पार्क में एक बच्चा नहीं था।</t>
+  </si>
+  <si>
+    <t>कल पार्क में कोई बच्चा नहीं था।</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>क्या आप यही चाहते थे?</t>
+  </si>
+  <si>
+    <t>Tom won't do that even if you ask him.</t>
+  </si>
+  <si>
+    <t>यदि तुम उसे पूछो तो भी टॉम उसे नहीं करेगा।</t>
+  </si>
+  <si>
+    <t>यदि तुम उसे पूछो भी टॉम उसे नहीं करेगा।</t>
+  </si>
+  <si>
+    <t>टॉम ऐसा नहीं करेगा, भले ही आप उससे पूछें।</t>
+  </si>
+  <si>
+    <t>even if</t>
+  </si>
+  <si>
+    <t>1801.mp3</t>
+  </si>
+  <si>
+    <t>47510.mp3</t>
+  </si>
+  <si>
+    <t>67306.mp3</t>
+  </si>
+  <si>
+    <t>244589.mp3</t>
+  </si>
+  <si>
+    <t>9419078.mp3</t>
   </si>
 </sst>
 </file>
@@ -478,11 +463,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -844,7 +830,7 @@
         <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>
@@ -873,7 +859,7 @@
         <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
@@ -902,7 +888,7 @@
         <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>122</v>
+        <v>93</v>
       </c>
       <c r="G4" t="s">
         <v>25</v>
@@ -931,7 +917,7 @@
         <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="G5" t="s">
         <v>30</v>
@@ -943,91 +929,91 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1283</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>108</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>35</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="H6" t="s">
         <v>15</v>
       </c>
       <c r="I6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1541</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
+        <v>43</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>113</v>
       </c>
       <c r="H7" t="s">
         <v>15</v>
       </c>
       <c r="I7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1018</v>
       </c>
       <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" t="s">
+        <v>117</v>
+      </c>
+      <c r="G8" t="s">
+        <v>119</v>
+      </c>
+      <c r="H8" t="s">
         <v>32</v>
       </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" t="s">
-        <v>126</v>
-      </c>
-      <c r="G8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" t="s">
-        <v>45</v>
-      </c>
       <c r="I8" t="s">
-        <v>46</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="87" x14ac:dyDescent="0.35">
@@ -1038,25 +1024,25 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="I9" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -1064,28 +1050,28 @@
         <v>1098</v>
       </c>
       <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" t="s">
         <v>32</v>
       </c>
-      <c r="C10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" t="s">
-        <v>128</v>
-      </c>
-      <c r="G10" t="s">
-        <v>55</v>
-      </c>
-      <c r="H10" t="s">
-        <v>45</v>
-      </c>
       <c r="I10" t="s">
-        <v>56</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -1096,25 +1082,25 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="F11" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="I11" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -1122,28 +1108,28 @@
         <v>1317</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="I12" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -1151,28 +1137,28 @@
         <v>17192</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="I13" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="203" x14ac:dyDescent="0.35">
@@ -1183,25 +1169,25 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="D14" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>132</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="I14" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="116" x14ac:dyDescent="0.35">
@@ -1212,54 +1198,54 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="G15" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="H15" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="304.5" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>724</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" t="s">
-        <v>83</v>
+        <v>43</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>127</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>85</v>
+        <v>129</v>
       </c>
       <c r="F16" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="G16" t="s">
-        <v>86</v>
+        <v>130</v>
       </c>
       <c r="H16" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="I16" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="217.5" x14ac:dyDescent="0.35">
@@ -1270,25 +1256,25 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" t="s">
         <v>90</v>
       </c>
-      <c r="F17" t="s">
-        <v>135</v>
-      </c>
-      <c r="G17" t="s">
-        <v>119</v>
-      </c>
       <c r="H17" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="I17" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="246.5" x14ac:dyDescent="0.35">
@@ -1299,25 +1285,25 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>102</v>
       </c>
       <c r="G18" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="H18" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="I18" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="87" x14ac:dyDescent="0.35">
@@ -1328,54 +1314,54 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="D19" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="G19" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="H19" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I19" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="116" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2560</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" t="s">
-        <v>103</v>
+        <v>43</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>79</v>
       </c>
       <c r="D20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" t="s">
         <v>104</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" t="s">
-        <v>138</v>
-      </c>
       <c r="G20" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="H20" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I20" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="58" x14ac:dyDescent="0.35">
@@ -1383,28 +1369,28 @@
         <v>392111</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="F21" t="s">
-        <v>139</v>
+        <v>104</v>
       </c>
       <c r="G21" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I21" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
@@ -1412,28 +1398,28 @@
         <v>2288136</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="F22" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="G22" t="s">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="H22" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I22" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>